<commit_message>
Apply glossary and Gantt label fixes (annex_2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBrdW2XtzbJ3UGSgGZS6cE
</commit_message>
<xml_diff>
--- a/Gantt_Guo_Zi_Qiang_Robin.xlsx
+++ b/Gantt_Guo_Zi_Qiang_Robin.xlsx
@@ -26,7 +26,7 @@
     <t xml:space="preserve">Gantt chart: AI Security for Critical Infrastructure (Guardrail Evaluation Test Bench and Beacon)</t>
   </si>
   <si>
-    <t xml:space="preserve">Guo Zi Qiang Robin, SIT AAI4001 Capstone at LTA (CYAD). Capstone period 8 Oct 2026 to 31 Mar 2027. Weekly columns start on the date shown and run Thursday to Wednesday. See the Legend sheet.</t>
+    <t xml:space="preserve">Guo Zi Qiang Robin, AAI4001 Capstone at LTA (CYAD). Capstone period 8 Oct 2026 to 31 Mar 2027. Weekly columns start on the date shown and run Thursday to Wednesday. See the Legend sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">Chart start date</t>
@@ -53,7 +53,7 @@
     <t xml:space="preserve">Deliverable</t>
   </si>
   <si>
-    <t xml:space="preserve">SIT milestones</t>
+    <t xml:space="preserve">Academic milestones</t>
   </si>
   <si>
     <t xml:space="preserve">Group</t>
@@ -77,7 +77,7 @@
     <t xml:space="preserve">Interim report (Form E1) submitted</t>
   </si>
   <si>
-    <t xml:space="preserve">Benchtest report; Tier 1 results</t>
+    <t xml:space="preserve">Test bench evaluation report; Tier 1 results</t>
   </si>
   <si>
     <t xml:space="preserve">Form E1</t>
@@ -92,7 +92,7 @@
     <t xml:space="preserve">Final report (Form E2) submitted</t>
   </si>
   <si>
-    <t xml:space="preserve">Deployed Beacon; benchtest report</t>
+    <t xml:space="preserve">Deployed Beacon; test bench evaluation report</t>
   </si>
   <si>
     <t xml:space="preserve">Form E2</t>
@@ -194,10 +194,10 @@
     <t xml:space="preserve">Results dataset</t>
   </si>
   <si>
-    <t xml:space="preserve">Write benchtest report</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benchtest report</t>
+    <t xml:space="preserve">Write test bench evaluation report</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test bench evaluation report</t>
   </si>
   <si>
     <t xml:space="preserve">Tidy harness, dataset and documentation</t>
@@ -1342,7 +1342,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
         <v>22</v>
       </c>

</xml_diff>